<commit_message>
feat: resultados reais, fixes simulação (λ, terceiros, sede, desempate)
</commit_message>
<xml_diff>
--- a/data/raw/Dados_Selecoes.xlsx
+++ b/data/raw/Dados_Selecoes.xlsx
@@ -574,7 +574,7 @@
         <v>3437</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="7">
@@ -622,7 +622,7 @@
         <v>3383</v>
       </c>
       <c r="F8" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="9">
@@ -670,7 +670,7 @@
         <v>3446</v>
       </c>
       <c r="F10" t="n">
-        <v>65</v>
+        <v>64</v>
       </c>
     </row>
     <row r="11">
@@ -718,7 +718,7 @@
         <v>4311</v>
       </c>
       <c r="F12" t="n">
-        <v>69</v>
+        <v>68</v>
       </c>
     </row>
     <row r="13">
@@ -838,7 +838,7 @@
         <v>3591</v>
       </c>
       <c r="F17" t="n">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="18">
@@ -886,7 +886,7 @@
         <v>32364</v>
       </c>
       <c r="F19" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="20">
@@ -934,7 +934,7 @@
         <v>5750</v>
       </c>
       <c r="F21" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="22">
@@ -1030,7 +1030,7 @@
         <v>3377</v>
       </c>
       <c r="F25" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="26">
@@ -1054,7 +1054,7 @@
         <v>3441</v>
       </c>
       <c r="F26" t="n">
-        <v>74</v>
+        <v>73</v>
       </c>
     </row>
     <row r="27">
@@ -1078,7 +1078,7 @@
         <v>14161</v>
       </c>
       <c r="F27" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="28">
@@ -1102,7 +1102,7 @@
         <v>3379</v>
       </c>
       <c r="F28" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29">
@@ -1150,7 +1150,7 @@
         <v>3582</v>
       </c>
       <c r="F30" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
     </row>
     <row r="31">
@@ -1174,7 +1174,7 @@
         <v>3560</v>
       </c>
       <c r="F31" t="n">
-        <v>57</v>
+        <v>56</v>
       </c>
     </row>
     <row r="32">
@@ -1246,7 +1246,7 @@
         <v>3575</v>
       </c>
       <c r="F34" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="35">
@@ -1270,7 +1270,7 @@
         <v>6303</v>
       </c>
       <c r="F35" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36">
@@ -1342,7 +1342,7 @@
         <v>3577</v>
       </c>
       <c r="F38" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="39">
@@ -1414,7 +1414,7 @@
         <v>3854</v>
       </c>
       <c r="F41" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="42">
@@ -1438,7 +1438,7 @@
         <v>3445</v>
       </c>
       <c r="F42" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="43">
@@ -1462,7 +1462,7 @@
         <v>3499</v>
       </c>
       <c r="F43" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="44">
@@ -1534,7 +1534,7 @@
         <v>3670</v>
       </c>
       <c r="F46" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="47">
@@ -1693,14 +1693,14 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>France</t>
+          <t>Argentina</t>
         </is>
       </c>
       <c r="B2" t="n">
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1877.32</v>
+        <v>1874.81</v>
       </c>
     </row>
     <row r="3">
@@ -1713,20 +1713,20 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>1876.4</v>
+        <v>1873.01</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Argentina</t>
+          <t>France</t>
         </is>
       </c>
       <c r="B4" t="n">
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>1874.81</v>
+        <v>1869.43</v>
       </c>
     </row>
     <row r="5">
@@ -1765,33 +1765,33 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>1761.16</v>
+        <v>1762.66</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Netherlands</t>
+          <t>Morocco</t>
         </is>
       </c>
       <c r="B8" t="n">
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>1757.87</v>
+        <v>1756.94</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Morocco</t>
+          <t>Netherlands</t>
         </is>
       </c>
       <c r="B9" t="n">
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>1755.87</v>
+        <v>1751.1</v>
       </c>
     </row>
     <row r="10">
@@ -1804,7 +1804,7 @@
         <v>9</v>
       </c>
       <c r="C10" t="n">
-        <v>1734.71</v>
+        <v>1742.24</v>
       </c>
     </row>
     <row r="11">
@@ -1817,7 +1817,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>1730.37</v>
+        <v>1731.3</v>
       </c>
     </row>
     <row r="12">
@@ -1830,7 +1830,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>1717.07</v>
+        <v>1712.24</v>
       </c>
     </row>
     <row r="13">
@@ -1843,7 +1843,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>1700.37</v>
+        <v>1701.77</v>
       </c>
     </row>
     <row r="14">
@@ -1856,33 +1856,33 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>1693.09</v>
+        <v>1695.99</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Senegal</t>
+          <t>Mexico</t>
         </is>
       </c>
       <c r="B15" t="n">
         <v>14</v>
       </c>
       <c r="C15" t="n">
-        <v>1688.99</v>
+        <v>1687.48</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Mexico</t>
+          <t>Senegal</t>
         </is>
       </c>
       <c r="B16" t="n">
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>1681.03</v>
+        <v>1686.41</v>
       </c>
     </row>
     <row r="17">
@@ -1895,7 +1895,7 @@
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>1673.13</v>
+        <v>1675.7</v>
       </c>
     </row>
     <row r="18">
@@ -1921,7 +1921,7 @@
         <v>18</v>
       </c>
       <c r="C19" t="n">
-        <v>1660.43</v>
+        <v>1661.58</v>
       </c>
     </row>
     <row r="20">
@@ -1934,33 +1934,33 @@
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>1649.4</v>
+        <v>1650.75</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Denmark</t>
+          <t>IR Iran</t>
         </is>
       </c>
       <c r="B21" t="n">
         <v>20</v>
       </c>
       <c r="C21" t="n">
-        <v>1620.81</v>
+        <v>1619.58</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IR Iran</t>
+          <t>Denmark</t>
         </is>
       </c>
       <c r="B22" t="n">
         <v>21</v>
       </c>
       <c r="C22" t="n">
-        <v>1615.3</v>
+        <v>1619.47</v>
       </c>
     </row>
     <row r="23">
@@ -1973,33 +1973,33 @@
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>1599.04</v>
+        <v>1601.99</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>1594.78</v>
+        <v>1597.4</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>1593.45</v>
+        <v>1596.48</v>
       </c>
     </row>
     <row r="26">
@@ -2012,7 +2012,7 @@
         <v>25</v>
       </c>
       <c r="C26" t="n">
-        <v>1588.66</v>
+        <v>1591.63</v>
       </c>
     </row>
     <row r="27">
@@ -2025,7 +2025,7 @@
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>1585.09</v>
+        <v>1586.69</v>
       </c>
     </row>
     <row r="28">
@@ -2038,7 +2038,7 @@
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>1580.67</v>
+        <v>1578.66</v>
       </c>
     </row>
     <row r="29">
@@ -2051,7 +2051,7 @@
         <v>28</v>
       </c>
       <c r="C29" t="n">
-        <v>1564.26</v>
+        <v>1571.03</v>
       </c>
     </row>
     <row r="30">
@@ -2064,7 +2064,7 @@
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>1563.24</v>
+        <v>1565.56</v>
       </c>
     </row>
     <row r="31">
@@ -2077,7 +2077,7 @@
         <v>30</v>
       </c>
       <c r="C31" t="n">
-        <v>1556.48</v>
+        <v>1559.48</v>
       </c>
     </row>
     <row r="32">
@@ -2090,7 +2090,7 @@
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>1550.94</v>
+        <v>1555.6</v>
       </c>
     </row>
     <row r="33">
@@ -2103,59 +2103,59 @@
         <v>32</v>
       </c>
       <c r="C33" t="n">
-        <v>1546.88</v>
+        <v>1549.29</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Panama</t>
+          <t>Côte d'Ivoire</t>
         </is>
       </c>
       <c r="B34" t="n">
         <v>33</v>
       </c>
       <c r="C34" t="n">
-        <v>1540.64</v>
+        <v>1540.87</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Côte d'Ivoire</t>
+          <t>Panama</t>
         </is>
       </c>
       <c r="B35" t="n">
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>1532.98</v>
+        <v>1540.6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Poland</t>
+          <t>Russia</t>
         </is>
       </c>
       <c r="B36" t="n">
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>1528</v>
+        <v>1527.24</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>Russia</t>
+          <t>Poland</t>
         </is>
       </c>
       <c r="B37" t="n">
         <v>36</v>
       </c>
       <c r="C37" t="n">
-        <v>1525.6</v>
+        <v>1526.18</v>
       </c>
     </row>
     <row r="38">
@@ -2168,7 +2168,7 @@
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>1524.29</v>
+        <v>1522.64</v>
       </c>
     </row>
     <row r="39">
@@ -2181,20 +2181,20 @@
         <v>38</v>
       </c>
       <c r="C39" t="n">
-        <v>1514.77</v>
+        <v>1509.79</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>1508.65</v>
+        <v>1505.74</v>
       </c>
     </row>
     <row r="41">
@@ -2207,33 +2207,33 @@
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>1503.5</v>
+        <v>1505.35</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>1501.38</v>
+        <v>1504.14</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>1500.58</v>
+        <v>1502.13</v>
       </c>
     </row>
     <row r="44">
@@ -2246,46 +2246,46 @@
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>1498.35</v>
+        <v>1499.92</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Cameroon</t>
         </is>
       </c>
       <c r="B45" t="n">
         <v>44</v>
       </c>
       <c r="C45" t="n">
-        <v>1483.05</v>
+        <v>1481.24</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Cameroon</t>
+          <t>Congo DR</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>1481.24</v>
+        <v>1479.68</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Congo DR</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>1478.35</v>
+        <v>1476.41</v>
       </c>
     </row>
     <row r="48">
@@ -2298,7 +2298,7 @@
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>1475.82</v>
+        <v>1476.15</v>
       </c>
     </row>
     <row r="49">
@@ -2311,7 +2311,7 @@
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>1473.94</v>
+        <v>1473.66</v>
       </c>
     </row>
     <row r="50">
@@ -2337,46 +2337,46 @@
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>1465.34</v>
+        <v>1461.21</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>1459.9</v>
+        <v>1459.39</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>1459.13</v>
+        <v>1457</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Mali</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>1455.87</v>
+        <v>1455.59</v>
       </c>
     </row>
     <row r="55">
@@ -2402,33 +2402,33 @@
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>1454.96</v>
+        <v>1452.37</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>1451.16</v>
+        <v>1451.15</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>1447.14</v>
+        <v>1450.2</v>
       </c>
     </row>
     <row r="59">
@@ -2441,7 +2441,7 @@
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>1446.44</v>
+        <v>1443.72</v>
       </c>
     </row>
     <row r="60">
@@ -2454,7 +2454,7 @@
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>1436.63</v>
+        <v>1441.1</v>
       </c>
     </row>
     <row r="61">
@@ -2467,7 +2467,7 @@
         <v>60</v>
       </c>
       <c r="C61" t="n">
-        <v>1429.73</v>
+        <v>1428.38</v>
       </c>
     </row>
     <row r="62">
@@ -2480,7 +2480,7 @@
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>1421.43</v>
+        <v>1421.54</v>
       </c>
     </row>
     <row r="63">
@@ -2493,7 +2493,7 @@
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>1412.49</v>
+        <v>1408.54</v>
       </c>
     </row>
     <row r="64">
@@ -2506,33 +2506,33 @@
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>1391.45</v>
+        <v>1390.1</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>Albania</t>
+          <t>Bosnia and Herzegovina</t>
         </is>
       </c>
       <c r="B65" t="n">
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>1388.06</v>
+        <v>1385.77</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Bosnia and Herzegovina</t>
+          <t>Albania</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>1385.84</v>
+        <v>1382.49</v>
       </c>
     </row>
     <row r="67">
@@ -2551,40 +2551,40 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>North Macedonia</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>1372.04</v>
+        <v>1370.47</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Cabo Verde</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>1370.47</v>
+        <v>1369.29</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>Cabo Verde</t>
+          <t>North Macedonia</t>
         </is>
       </c>
       <c r="B70" t="n">
         <v>69</v>
       </c>
       <c r="C70" t="n">
-        <v>1366.13</v>
+        <v>1369.16</v>
       </c>
     </row>
     <row r="71">
@@ -2597,7 +2597,7 @@
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>1362.16</v>
+        <v>1366.56</v>
       </c>
     </row>
     <row r="72">
@@ -2610,7 +2610,7 @@
         <v>71</v>
       </c>
       <c r="C72" t="n">
-        <v>1358</v>
+        <v>1357.84</v>
       </c>
     </row>
     <row r="73">
@@ -2623,72 +2623,72 @@
         <v>72</v>
       </c>
       <c r="C73" t="n">
-        <v>1350.18</v>
+        <v>1355.26</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>Finland</t>
+          <t>Ghana</t>
         </is>
       </c>
       <c r="B74" t="n">
         <v>73</v>
       </c>
       <c r="C74" t="n">
-        <v>1346.41</v>
+        <v>1346.88</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>Ghana</t>
+          <t>Iceland</t>
         </is>
       </c>
       <c r="B75" t="n">
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>1346.31</v>
+        <v>1343.92</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>Iceland</t>
+          <t>Finland</t>
         </is>
       </c>
       <c r="B76" t="n">
         <v>75</v>
       </c>
       <c r="C76" t="n">
-        <v>1345.07</v>
+        <v>1341.92</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>Bolivia</t>
+          <t>Israel</t>
         </is>
       </c>
       <c r="B77" t="n">
         <v>76</v>
       </c>
       <c r="C77" t="n">
-        <v>1329.42</v>
+        <v>1333.9</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>Israel</t>
+          <t>Bolivia</t>
         </is>
       </c>
       <c r="B78" t="n">
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>1328.33</v>
+        <v>1329.42</v>
       </c>
     </row>
     <row r="79">
@@ -2701,7 +2701,7 @@
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>1318.83</v>
+        <v>1317.17</v>
       </c>
     </row>
     <row r="80">
@@ -2714,59 +2714,59 @@
         <v>79</v>
       </c>
       <c r="C80" t="n">
-        <v>1313.46</v>
+        <v>1306.9</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>Guinea</t>
+          <t>Montenegro</t>
         </is>
       </c>
       <c r="B81" t="n">
         <v>80</v>
       </c>
       <c r="C81" t="n">
-        <v>1300.01</v>
+        <v>1301.98</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>Montenegro</t>
+          <t>Guinea</t>
         </is>
       </c>
       <c r="B82" t="n">
         <v>81</v>
       </c>
       <c r="C82" t="n">
-        <v>1295.52</v>
+        <v>1295.6</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>1294.65</v>
+        <v>1293.1</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>1291.71</v>
+        <v>1293.08</v>
       </c>
     </row>
     <row r="85">
@@ -2779,7 +2779,7 @@
         <v>84</v>
       </c>
       <c r="C85" t="n">
-        <v>1288.56</v>
+        <v>1283.05</v>
       </c>
     </row>
     <row r="86">
@@ -2792,33 +2792,33 @@
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>1281.57</v>
+        <v>1276.66</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>Bulgaria</t>
+          <t>Gabon</t>
         </is>
       </c>
       <c r="B87" t="n">
         <v>86</v>
       </c>
       <c r="C87" t="n">
-        <v>1278.9</v>
+        <v>1272.51</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>Gabon</t>
+          <t>Bulgaria</t>
         </is>
       </c>
       <c r="B88" t="n">
         <v>87</v>
       </c>
       <c r="C88" t="n">
-        <v>1272.51</v>
+        <v>1271.68</v>
       </c>
     </row>
     <row r="89">
@@ -2844,7 +2844,7 @@
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>1263.1</v>
+        <v>1262.22</v>
       </c>
     </row>
     <row r="91">
@@ -2857,59 +2857,59 @@
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>1258.98</v>
+        <v>1258.22</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>1258.53</v>
+        <v>1255.82</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>China PR</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>1255.82</v>
+        <v>1254.85</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Thailand</t>
+          <t>Bahrain</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>1252.14</v>
+        <v>1254.41</v>
       </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>China PR</t>
+          <t>Thailand</t>
         </is>
       </c>
       <c r="B95" t="n">
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>1251.6</v>
+        <v>1250.76</v>
       </c>
     </row>
     <row r="96">
@@ -2928,27 +2928,27 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>Guatemala</t>
+          <t>Belarus</t>
         </is>
       </c>
       <c r="B97" t="n">
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>1243.47</v>
+        <v>1241.32</v>
       </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>Belarus</t>
+          <t>Guatemala</t>
         </is>
       </c>
       <c r="B98" t="n">
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>1235.82</v>
+        <v>1240.78</v>
       </c>
     </row>
     <row r="99">
@@ -2961,7 +2961,7 @@
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>1227.77</v>
+        <v>1226.36</v>
       </c>
     </row>
     <row r="100">
@@ -2980,14 +2980,14 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>El Salvador</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>1225.26</v>
+        <v>1225.52</v>
       </c>
     </row>
     <row r="102">
@@ -3006,27 +3006,27 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>Trinidad and Tobago</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="B103" t="n">
         <v>102</v>
       </c>
       <c r="C103" t="n">
-        <v>1222.94</v>
+        <v>1223.28</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>Trinidad and Tobago</t>
         </is>
       </c>
       <c r="B104" t="n">
         <v>103</v>
       </c>
       <c r="C104" t="n">
-        <v>1221.78</v>
+        <v>1221.95</v>
       </c>
     </row>
     <row r="105">
@@ -3039,7 +3039,7 @@
         <v>104</v>
       </c>
       <c r="C105" t="n">
-        <v>1203.76</v>
+        <v>1202.69</v>
       </c>
     </row>
     <row r="106">
@@ -3065,7 +3065,7 @@
         <v>106</v>
       </c>
       <c r="C107" t="n">
-        <v>1191.42</v>
+        <v>1191.33</v>
       </c>
     </row>
     <row r="108">
@@ -3084,40 +3084,40 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Comoros</t>
         </is>
       </c>
       <c r="B109" t="n">
         <v>108</v>
       </c>
       <c r="C109" t="n">
-        <v>1187.96</v>
+        <v>1187.91</v>
       </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Comoros</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B110" t="n">
         <v>109</v>
       </c>
       <c r="C110" t="n">
-        <v>1187.91</v>
+        <v>1183.04</v>
       </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Libya</t>
         </is>
       </c>
       <c r="B111" t="n">
         <v>110</v>
       </c>
       <c r="C111" t="n">
-        <v>1182.96</v>
+        <v>1182.08</v>
       </c>
     </row>
     <row r="112">
@@ -3130,20 +3130,20 @@
         <v>111</v>
       </c>
       <c r="C112" t="n">
-        <v>1182.23</v>
+        <v>1181.14</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Libya</t>
+          <t>Niger</t>
         </is>
       </c>
       <c r="B113" t="n">
         <v>112</v>
       </c>
       <c r="C113" t="n">
-        <v>1182.08</v>
+        <v>1180.42</v>
       </c>
     </row>
     <row r="114">
@@ -3162,14 +3162,14 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Niger</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B115" t="n">
         <v>114</v>
       </c>
       <c r="C115" t="n">
-        <v>1179.66</v>
+        <v>1172.22</v>
       </c>
     </row>
     <row r="116">
@@ -3182,7 +3182,7 @@
         <v>115</v>
       </c>
       <c r="C116" t="n">
-        <v>1170.72</v>
+        <v>1171.6</v>
       </c>
     </row>
     <row r="117">
@@ -3195,7 +3195,7 @@
         <v>116</v>
       </c>
       <c r="C117" t="n">
-        <v>1160.38</v>
+        <v>1159.64</v>
       </c>
     </row>
     <row r="118">
@@ -3214,66 +3214,66 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>Korea DPR</t>
+          <t>Indonesia</t>
         </is>
       </c>
       <c r="B119" t="n">
         <v>118</v>
       </c>
       <c r="C119" t="n">
-        <v>1151.05</v>
+        <v>1151.45</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Sierra Leone</t>
+          <t>Korea DPR</t>
         </is>
       </c>
       <c r="B120" t="n">
         <v>119</v>
       </c>
       <c r="C120" t="n">
-        <v>1148.98</v>
+        <v>1151.05</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Namibia</t>
+          <t>Sierra Leone</t>
         </is>
       </c>
       <c r="B121" t="n">
         <v>120</v>
       </c>
       <c r="C121" t="n">
-        <v>1148.84</v>
+        <v>1148.98</v>
       </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>Togo</t>
+          <t>Namibia</t>
         </is>
       </c>
       <c r="B122" t="n">
         <v>121</v>
       </c>
       <c r="C122" t="n">
-        <v>1147.31</v>
+        <v>1148.84</v>
       </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Indonesia</t>
+          <t>Togo</t>
         </is>
       </c>
       <c r="B123" t="n">
         <v>122</v>
       </c>
       <c r="C123" t="n">
-        <v>1144.88</v>
+        <v>1146.7</v>
       </c>
     </row>
     <row r="124">
@@ -3292,40 +3292,40 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Azerbaijan</t>
+          <t>Suriname</t>
         </is>
       </c>
       <c r="B125" t="n">
         <v>124</v>
       </c>
       <c r="C125" t="n">
-        <v>1136.67</v>
+        <v>1132.43</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Suriname</t>
+          <t>Cyprus</t>
         </is>
       </c>
       <c r="B126" t="n">
         <v>125</v>
       </c>
       <c r="C126" t="n">
-        <v>1132.43</v>
+        <v>1131.06</v>
       </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>Cyprus</t>
+          <t>Azerbaijan</t>
         </is>
       </c>
       <c r="B127" t="n">
         <v>126</v>
       </c>
       <c r="C127" t="n">
-        <v>1128.33</v>
+        <v>1130.26</v>
       </c>
     </row>
     <row r="128">
@@ -3377,7 +3377,7 @@
         <v>130</v>
       </c>
       <c r="C131" t="n">
-        <v>1118.12</v>
+        <v>1119.78</v>
       </c>
     </row>
     <row r="132">
@@ -3390,7 +3390,7 @@
         <v>131</v>
       </c>
       <c r="C132" t="n">
-        <v>1115.13</v>
+        <v>1114.63</v>
       </c>
     </row>
     <row r="133">
@@ -3409,27 +3409,27 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>Congo</t>
+          <t>Kuwait</t>
         </is>
       </c>
       <c r="B134" t="n">
         <v>133</v>
       </c>
       <c r="C134" t="n">
-        <v>1105.96</v>
+        <v>1106.47</v>
       </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>Kuwait</t>
+          <t>Congo</t>
         </is>
       </c>
       <c r="B135" t="n">
         <v>134</v>
       </c>
       <c r="C135" t="n">
-        <v>1105.1</v>
+        <v>1105.96</v>
       </c>
     </row>
     <row r="136">
@@ -3442,59 +3442,59 @@
         <v>135</v>
       </c>
       <c r="C136" t="n">
-        <v>1094.1</v>
+        <v>1096.73</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B137" t="n">
         <v>136</v>
       </c>
       <c r="C137" t="n">
-        <v>1091.03</v>
+        <v>1090.57</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="B138" t="n">
         <v>137</v>
       </c>
       <c r="C138" t="n">
-        <v>1090.57</v>
+        <v>1086.22</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Central African Republic</t>
         </is>
       </c>
       <c r="B139" t="n">
         <v>138</v>
       </c>
       <c r="C139" t="n">
-        <v>1086.22</v>
+        <v>1084.18</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>Central African Republic</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B140" t="n">
         <v>139</v>
       </c>
       <c r="C140" t="n">
-        <v>1083.57</v>
+        <v>1083.6</v>
       </c>
     </row>
     <row r="141">
@@ -3546,7 +3546,7 @@
         <v>143</v>
       </c>
       <c r="C144" t="n">
-        <v>1077.95</v>
+        <v>1076.5</v>
       </c>
     </row>
     <row r="145">
@@ -3572,33 +3572,33 @@
         <v>145</v>
       </c>
       <c r="C146" t="n">
-        <v>1067.13</v>
+        <v>1068.22</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Botswana</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="B147" t="n">
         <v>146</v>
       </c>
       <c r="C147" t="n">
-        <v>1063.63</v>
+        <v>1065.24</v>
       </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Botswana</t>
         </is>
       </c>
       <c r="B148" t="n">
         <v>147</v>
       </c>
       <c r="C148" t="n">
-        <v>1059.53</v>
+        <v>1063.63</v>
       </c>
     </row>
     <row r="149">
@@ -3617,14 +3617,14 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Yemen</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="B150" t="n">
         <v>149</v>
       </c>
       <c r="C150" t="n">
-        <v>1049.49</v>
+        <v>1057.95</v>
       </c>
     </row>
     <row r="151">
@@ -3682,27 +3682,27 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Fiji</t>
+          <t>Hong Kong, China</t>
         </is>
       </c>
       <c r="B155" t="n">
         <v>154</v>
       </c>
       <c r="C155" t="n">
-        <v>1029.7</v>
+        <v>1030.24</v>
       </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>Hong Kong, China</t>
+          <t>Fiji</t>
         </is>
       </c>
       <c r="B156" t="n">
         <v>155</v>
       </c>
       <c r="C156" t="n">
-        <v>1026.63</v>
+        <v>1024.38</v>
       </c>
     </row>
     <row r="157">
@@ -3715,7 +3715,7 @@
         <v>156</v>
       </c>
       <c r="C157" t="n">
-        <v>1026.11</v>
+        <v>1024.3</v>
       </c>
     </row>
     <row r="158">
@@ -3754,7 +3754,7 @@
         <v>159</v>
       </c>
       <c r="C160" t="n">
-        <v>1004.16</v>
+        <v>1006.54</v>
       </c>
     </row>
     <row r="161">
@@ -3767,7 +3767,7 @@
         <v>160</v>
       </c>
       <c r="C161" t="n">
-        <v>997.01</v>
+        <v>1002.32</v>
       </c>
     </row>
     <row r="162">
@@ -3780,7 +3780,7 @@
         <v>161</v>
       </c>
       <c r="C162" t="n">
-        <v>987.73</v>
+        <v>992.79</v>
       </c>
     </row>
     <row r="163">
@@ -3806,7 +3806,7 @@
         <v>163</v>
       </c>
       <c r="C164" t="n">
-        <v>982.5700000000001</v>
+        <v>981.8200000000001</v>
       </c>
     </row>
     <row r="165">
@@ -3838,53 +3838,53 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Bermuda</t>
+          <t>Afghanistan</t>
         </is>
       </c>
       <c r="B167" t="n">
         <v>166</v>
       </c>
       <c r="C167" t="n">
-        <v>976.87</v>
+        <v>977.5700000000001</v>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>St Lucia</t>
+          <t>Bermuda</t>
         </is>
       </c>
       <c r="B168" t="n">
         <v>167</v>
       </c>
       <c r="C168" t="n">
-        <v>976.71</v>
+        <v>976.87</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>Papua New Guinea</t>
+          <t>St Lucia</t>
         </is>
       </c>
       <c r="B169" t="n">
         <v>168</v>
       </c>
       <c r="C169" t="n">
-        <v>974.9</v>
+        <v>976.71</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Afghanistan</t>
+          <t>Papua New Guinea</t>
         </is>
       </c>
       <c r="B170" t="n">
         <v>169</v>
       </c>
       <c r="C170" t="n">
-        <v>972.75</v>
+        <v>974.9</v>
       </c>
     </row>
     <row r="171">
@@ -3916,27 +3916,27 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>Maldives</t>
+          <t>Andorra</t>
         </is>
       </c>
       <c r="B173" t="n">
         <v>172</v>
       </c>
       <c r="C173" t="n">
-        <v>954.9299999999999</v>
+        <v>948.38</v>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>Andorra</t>
+          <t>Maldives</t>
         </is>
       </c>
       <c r="B174" t="n">
         <v>173</v>
       </c>
       <c r="C174" t="n">
-        <v>945.34</v>
+        <v>943.92</v>
       </c>
     </row>
     <row r="175">
@@ -3968,27 +3968,27 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Nepal</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="B177" t="n">
         <v>176</v>
       </c>
       <c r="C177" t="n">
-        <v>914.54</v>
+        <v>916.24</v>
       </c>
     </row>
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Nepal</t>
         </is>
       </c>
       <c r="B178" t="n">
         <v>177</v>
       </c>
       <c r="C178" t="n">
-        <v>911.54</v>
+        <v>914.54</v>
       </c>
     </row>
     <row r="179">
@@ -4040,7 +4040,7 @@
         <v>181</v>
       </c>
       <c r="C182" t="n">
-        <v>899.53</v>
+        <v>902.9299999999999</v>
       </c>
     </row>
     <row r="183">
@@ -4098,66 +4098,66 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>Cook Islands</t>
         </is>
       </c>
       <c r="B187" t="n">
         <v>186</v>
       </c>
       <c r="C187" t="n">
-        <v>880.55</v>
+        <v>877.53</v>
       </c>
     </row>
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Mongolia</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B188" t="n">
         <v>187</v>
       </c>
       <c r="C188" t="n">
-        <v>879.75</v>
+        <v>877.3</v>
       </c>
     </row>
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>Cook Islands</t>
+          <t>Samoa</t>
         </is>
       </c>
       <c r="B189" t="n">
         <v>188</v>
       </c>
       <c r="C189" t="n">
-        <v>877.53</v>
+        <v>876.41</v>
       </c>
     </row>
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Aruba</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="B190" t="n">
         <v>189</v>
       </c>
       <c r="C190" t="n">
-        <v>877.3</v>
+        <v>875.85</v>
       </c>
     </row>
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>Samoa</t>
+          <t>Mongolia</t>
         </is>
       </c>
       <c r="B191" t="n">
         <v>190</v>
       </c>
       <c r="C191" t="n">
-        <v>876.41</v>
+        <v>874.47</v>
       </c>
     </row>
     <row r="192">
@@ -4280,40 +4280,40 @@
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Timor-Leste</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="B201" t="n">
         <v>200</v>
       </c>
       <c r="C201" t="n">
-        <v>825.64</v>
+        <v>830.78</v>
       </c>
     </row>
     <row r="202">
       <c r="A202" t="inlineStr">
         <is>
-          <t>Guam</t>
+          <t>Timor-Leste</t>
         </is>
       </c>
       <c r="B202" t="n">
         <v>201</v>
       </c>
       <c r="C202" t="n">
-        <v>825.4299999999999</v>
+        <v>825.64</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Guam</t>
         </is>
       </c>
       <c r="B203" t="n">
         <v>202</v>
       </c>
       <c r="C203" t="n">
-        <v>824.6</v>
+        <v>822.8</v>
       </c>
     </row>
     <row r="204">
@@ -4326,7 +4326,7 @@
         <v>203</v>
       </c>
       <c r="C204" t="n">
-        <v>810.14</v>
+        <v>814.87</v>
       </c>
     </row>
     <row r="205">
@@ -4365,7 +4365,7 @@
         <v>206</v>
       </c>
       <c r="C207" t="n">
-        <v>803.5700000000001</v>
+        <v>799.89</v>
       </c>
     </row>
     <row r="208">
@@ -4384,27 +4384,27 @@
     <row r="209">
       <c r="A209" t="inlineStr">
         <is>
-          <t>British Virgin Islands</t>
+          <t>US Virgin Islands</t>
         </is>
       </c>
       <c r="B209" t="n">
         <v>208</v>
       </c>
       <c r="C209" t="n">
-        <v>782.14</v>
+        <v>779.76</v>
       </c>
     </row>
     <row r="210">
       <c r="A210" t="inlineStr">
         <is>
-          <t>US Virgin Islands</t>
+          <t>British Virgin Islands</t>
         </is>
       </c>
       <c r="B210" t="n">
         <v>209</v>
       </c>
       <c r="C210" t="n">
-        <v>779.76</v>
+        <v>777.41</v>
       </c>
     </row>
     <row r="211">
@@ -4430,7 +4430,7 @@
         <v>211</v>
       </c>
       <c r="C212" t="n">
-        <v>726.33</v>
+        <v>722.9299999999999</v>
       </c>
     </row>
   </sheetData>
@@ -4576,7 +4576,7 @@
     </row>
     <row r="6">
       <c r="A6" s="1" t="n">
-        <v>46186.04166666666</v>
+        <v>46187.04166666666</v>
       </c>
       <c r="B6" t="inlineStr">
         <is>
@@ -5080,7 +5080,7 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Atlanta</t>
+          <t>Akron</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
@@ -5155,7 +5155,7 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Akron</t>
+          <t>Atlanta</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
@@ -5176,7 +5176,7 @@
     </row>
     <row r="30">
       <c r="A30" s="1" t="n">
-        <v>46192.04166666666</v>
+        <v>46193.04166666666</v>
       </c>
       <c r="B30" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
feat: atualização simulação 11/06 + fase eliminatória nos resultados reais
- Atualiza dados de ranking FIFA, simulação e histórico (11/06/2026)
- Implementa acompanhamento da fase eliminatória na aba Resultados Reais:
  entrada de resultados para R16, Oitavas, Quartas, Semis, Final e 3º lugar;
  resolução automática dos times via classificação real dos grupos;
  suporte a prorrogação e pênaltis; comparação com Meu Cenário nos acertos

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/raw/Dados_Selecoes.xlsx
+++ b/data/raw/Dados_Selecoes.xlsx
@@ -622,7 +622,7 @@
         <v>3383</v>
       </c>
       <c r="F8" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="9">
@@ -718,7 +718,7 @@
         <v>4311</v>
       </c>
       <c r="F12" t="n">
-        <v>68</v>
+        <v>67</v>
       </c>
     </row>
     <row r="13">
@@ -766,7 +766,7 @@
         <v>14162</v>
       </c>
       <c r="F14" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="15">
@@ -886,7 +886,7 @@
         <v>32364</v>
       </c>
       <c r="F19" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="20">
@@ -934,7 +934,7 @@
         <v>5750</v>
       </c>
       <c r="F21" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
     </row>
     <row r="22">
@@ -958,7 +958,7 @@
         <v>3380</v>
       </c>
       <c r="F22" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23">
@@ -1006,7 +1006,7 @@
         <v>3505</v>
       </c>
       <c r="F24" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="25">
@@ -1078,7 +1078,7 @@
         <v>14161</v>
       </c>
       <c r="F27" t="n">
-        <v>82</v>
+        <v>83</v>
       </c>
     </row>
     <row r="28">
@@ -1174,7 +1174,7 @@
         <v>3560</v>
       </c>
       <c r="F31" t="n">
-        <v>56</v>
+        <v>57</v>
       </c>
     </row>
     <row r="32">
@@ -1366,7 +1366,7 @@
         <v>3581</v>
       </c>
       <c r="F39" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40">
@@ -1414,7 +1414,7 @@
         <v>3854</v>
       </c>
       <c r="F41" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="42">
@@ -1438,7 +1438,7 @@
         <v>3445</v>
       </c>
       <c r="F42" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
     </row>
     <row r="43">
@@ -1534,7 +1534,7 @@
         <v>3670</v>
       </c>
       <c r="F46" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="47">
@@ -1582,7 +1582,7 @@
         <v>3449</v>
       </c>
       <c r="F48" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
     </row>
     <row r="49">
@@ -1700,7 +1700,7 @@
         <v>1</v>
       </c>
       <c r="C2" t="n">
-        <v>1874.81</v>
+        <v>1877.27</v>
       </c>
     </row>
     <row r="3">
@@ -1713,7 +1713,7 @@
         <v>2</v>
       </c>
       <c r="C3" t="n">
-        <v>1873.01</v>
+        <v>1874.71</v>
       </c>
     </row>
     <row r="4">
@@ -1726,7 +1726,7 @@
         <v>3</v>
       </c>
       <c r="C4" t="n">
-        <v>1869.43</v>
+        <v>1870.7</v>
       </c>
     </row>
     <row r="5">
@@ -1739,7 +1739,7 @@
         <v>4</v>
       </c>
       <c r="C5" t="n">
-        <v>1825.97</v>
+        <v>1828.02</v>
       </c>
     </row>
     <row r="6">
@@ -1752,7 +1752,7 @@
         <v>5</v>
       </c>
       <c r="C6" t="n">
-        <v>1763.83</v>
+        <v>1767.85</v>
       </c>
     </row>
     <row r="7">
@@ -1765,7 +1765,7 @@
         <v>6</v>
       </c>
       <c r="C7" t="n">
-        <v>1762.66</v>
+        <v>1765.86</v>
       </c>
     </row>
     <row r="8">
@@ -1778,7 +1778,7 @@
         <v>7</v>
       </c>
       <c r="C8" t="n">
-        <v>1756.94</v>
+        <v>1755.1</v>
       </c>
     </row>
     <row r="9">
@@ -1791,7 +1791,7 @@
         <v>8</v>
       </c>
       <c r="C9" t="n">
-        <v>1751.1</v>
+        <v>1753.57</v>
       </c>
     </row>
     <row r="10">
@@ -1817,7 +1817,7 @@
         <v>10</v>
       </c>
       <c r="C11" t="n">
-        <v>1731.3</v>
+        <v>1735.77</v>
       </c>
     </row>
     <row r="12">
@@ -1830,7 +1830,7 @@
         <v>11</v>
       </c>
       <c r="C12" t="n">
-        <v>1712.24</v>
+        <v>1714.87</v>
       </c>
     </row>
     <row r="13">
@@ -1843,7 +1843,7 @@
         <v>12</v>
       </c>
       <c r="C13" t="n">
-        <v>1701.77</v>
+        <v>1704.73</v>
       </c>
     </row>
     <row r="14">
@@ -1856,7 +1856,7 @@
         <v>13</v>
       </c>
       <c r="C14" t="n">
-        <v>1695.99</v>
+        <v>1698.35</v>
       </c>
     </row>
     <row r="15">
@@ -1882,33 +1882,33 @@
         <v>15</v>
       </c>
       <c r="C16" t="n">
-        <v>1686.41</v>
+        <v>1684.07</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>USA</t>
+          <t>Uruguay</t>
         </is>
       </c>
       <c r="B17" t="n">
         <v>16</v>
       </c>
       <c r="C17" t="n">
-        <v>1675.7</v>
+        <v>1673.07</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>Uruguay</t>
+          <t>USA</t>
         </is>
       </c>
       <c r="B18" t="n">
         <v>17</v>
       </c>
       <c r="C18" t="n">
-        <v>1673.07</v>
+        <v>1671.23</v>
       </c>
     </row>
     <row r="19">
@@ -1934,7 +1934,7 @@
         <v>19</v>
       </c>
       <c r="C20" t="n">
-        <v>1650.75</v>
+        <v>1650.06</v>
       </c>
     </row>
     <row r="21">
@@ -1973,33 +1973,33 @@
         <v>22</v>
       </c>
       <c r="C23" t="n">
-        <v>1601.99</v>
+        <v>1605.73</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>Austria</t>
+          <t>Ecuador</t>
         </is>
       </c>
       <c r="B24" t="n">
         <v>23</v>
       </c>
       <c r="C24" t="n">
-        <v>1597.4</v>
+        <v>1598.52</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>Ecuador</t>
+          <t>Austria</t>
         </is>
       </c>
       <c r="B25" t="n">
         <v>24</v>
       </c>
       <c r="C25" t="n">
-        <v>1596.48</v>
+        <v>1597.4</v>
       </c>
     </row>
     <row r="26">
@@ -2025,7 +2025,7 @@
         <v>26</v>
       </c>
       <c r="C27" t="n">
-        <v>1586.69</v>
+        <v>1585.02</v>
       </c>
     </row>
     <row r="28">
@@ -2038,7 +2038,7 @@
         <v>27</v>
       </c>
       <c r="C28" t="n">
-        <v>1578.66</v>
+        <v>1579.34</v>
       </c>
     </row>
     <row r="29">
@@ -2064,7 +2064,7 @@
         <v>29</v>
       </c>
       <c r="C30" t="n">
-        <v>1565.56</v>
+        <v>1562.37</v>
       </c>
     </row>
     <row r="31">
@@ -2090,7 +2090,7 @@
         <v>31</v>
       </c>
       <c r="C32" t="n">
-        <v>1555.6</v>
+        <v>1557.44</v>
       </c>
     </row>
     <row r="33">
@@ -2129,7 +2129,7 @@
         <v>34</v>
       </c>
       <c r="C35" t="n">
-        <v>1540.6</v>
+        <v>1539.16</v>
       </c>
     </row>
     <row r="36">
@@ -2142,7 +2142,7 @@
         <v>35</v>
       </c>
       <c r="C36" t="n">
-        <v>1527.24</v>
+        <v>1529.6</v>
       </c>
     </row>
     <row r="37">
@@ -2168,7 +2168,7 @@
         <v>37</v>
       </c>
       <c r="C38" t="n">
-        <v>1522.64</v>
+        <v>1516.95</v>
       </c>
     </row>
     <row r="39">
@@ -2187,66 +2187,66 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>Czechia</t>
+          <t>Hungary</t>
         </is>
       </c>
       <c r="B40" t="n">
         <v>39</v>
       </c>
       <c r="C40" t="n">
-        <v>1505.74</v>
+        <v>1506.39</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>Paraguay</t>
+          <t>Czechia</t>
         </is>
       </c>
       <c r="B41" t="n">
         <v>40</v>
       </c>
       <c r="C41" t="n">
-        <v>1505.35</v>
+        <v>1505.74</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>Hungary</t>
+          <t>Paraguay</t>
         </is>
       </c>
       <c r="B42" t="n">
         <v>41</v>
       </c>
       <c r="C42" t="n">
-        <v>1504.14</v>
+        <v>1505.35</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Serbia</t>
+          <t>Scotland</t>
         </is>
       </c>
       <c r="B43" t="n">
         <v>42</v>
       </c>
       <c r="C43" t="n">
-        <v>1502.13</v>
+        <v>1503.34</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Scotland</t>
+          <t>Serbia</t>
         </is>
       </c>
       <c r="B44" t="n">
         <v>43</v>
       </c>
       <c r="C44" t="n">
-        <v>1499.92</v>
+        <v>1502.13</v>
       </c>
     </row>
     <row r="45">
@@ -2265,53 +2265,53 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Congo DR</t>
+          <t>Tunisia</t>
         </is>
       </c>
       <c r="B46" t="n">
         <v>45</v>
       </c>
       <c r="C46" t="n">
-        <v>1479.68</v>
+        <v>1476.41</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>Tunisia</t>
+          <t>Congo DR</t>
         </is>
       </c>
       <c r="B47" t="n">
         <v>46</v>
       </c>
       <c r="C47" t="n">
-        <v>1476.41</v>
+        <v>1474.43</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>Greece</t>
+          <t>Slovakia</t>
         </is>
       </c>
       <c r="B48" t="n">
         <v>47</v>
       </c>
       <c r="C48" t="n">
-        <v>1476.15</v>
+        <v>1473.66</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>Slovakia</t>
+          <t>Greece</t>
         </is>
       </c>
       <c r="B49" t="n">
         <v>48</v>
       </c>
       <c r="C49" t="n">
-        <v>1473.66</v>
+        <v>1473.19</v>
       </c>
     </row>
     <row r="50">
@@ -2324,7 +2324,7 @@
         <v>49</v>
       </c>
       <c r="C50" t="n">
-        <v>1468.05</v>
+        <v>1469.18</v>
       </c>
     </row>
     <row r="51">
@@ -2337,124 +2337,124 @@
         <v>50</v>
       </c>
       <c r="C51" t="n">
-        <v>1461.21</v>
+        <v>1458.73</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Peru</t>
+          <t>Chile</t>
         </is>
       </c>
       <c r="B52" t="n">
         <v>51</v>
       </c>
       <c r="C52" t="n">
-        <v>1459.39</v>
+        <v>1458.2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Costa Rica</t>
+          <t>Peru</t>
         </is>
       </c>
       <c r="B53" t="n">
         <v>52</v>
       </c>
       <c r="C53" t="n">
-        <v>1457</v>
+        <v>1457.69</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>Mali</t>
+          <t>Costa Rica</t>
         </is>
       </c>
       <c r="B54" t="n">
         <v>53</v>
       </c>
       <c r="C54" t="n">
-        <v>1455.59</v>
+        <v>1456.03</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>Chile</t>
+          <t>Romania</t>
         </is>
       </c>
       <c r="B55" t="n">
         <v>54</v>
       </c>
       <c r="C55" t="n">
-        <v>1455.28</v>
+        <v>1455.89</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>Qatar</t>
+          <t>Mali</t>
         </is>
       </c>
       <c r="B56" t="n">
         <v>55</v>
       </c>
       <c r="C56" t="n">
-        <v>1452.37</v>
+        <v>1455.59</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>Iraq</t>
+          <t>Qatar</t>
         </is>
       </c>
       <c r="B57" t="n">
         <v>56</v>
       </c>
       <c r="C57" t="n">
-        <v>1451.15</v>
+        <v>1450.31</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>Romania</t>
+          <t>Iraq</t>
         </is>
       </c>
       <c r="B58" t="n">
         <v>57</v>
       </c>
       <c r="C58" t="n">
-        <v>1450.2</v>
+        <v>1446.28</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>Slovenia</t>
+          <t>Republic of Ireland</t>
         </is>
       </c>
       <c r="B59" t="n">
         <v>58</v>
       </c>
       <c r="C59" t="n">
-        <v>1443.72</v>
+        <v>1441.1</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>Republic of Ireland</t>
+          <t>Slovenia</t>
         </is>
       </c>
       <c r="B60" t="n">
         <v>59</v>
       </c>
       <c r="C60" t="n">
-        <v>1441.1</v>
+        <v>1441.09</v>
       </c>
     </row>
     <row r="61">
@@ -2480,7 +2480,7 @@
         <v>61</v>
       </c>
       <c r="C62" t="n">
-        <v>1421.54</v>
+        <v>1423.88</v>
       </c>
     </row>
     <row r="63">
@@ -2493,7 +2493,7 @@
         <v>62</v>
       </c>
       <c r="C63" t="n">
-        <v>1408.54</v>
+        <v>1406.99</v>
       </c>
     </row>
     <row r="64">
@@ -2506,7 +2506,7 @@
         <v>63</v>
       </c>
       <c r="C64" t="n">
-        <v>1390.1</v>
+        <v>1387.74</v>
       </c>
     </row>
     <row r="65">
@@ -2519,59 +2519,59 @@
         <v>64</v>
       </c>
       <c r="C65" t="n">
-        <v>1385.77</v>
+        <v>1387.22</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>Albania</t>
+          <t>Honduras</t>
         </is>
       </c>
       <c r="B66" t="n">
         <v>65</v>
       </c>
       <c r="C66" t="n">
-        <v>1382.49</v>
+        <v>1378.97</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>Honduras</t>
+          <t>Albania</t>
         </is>
       </c>
       <c r="B67" t="n">
         <v>66</v>
       </c>
       <c r="C67" t="n">
-        <v>1380.27</v>
+        <v>1376.03</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>United Arab Emirates</t>
+          <t>Cabo Verde</t>
         </is>
       </c>
       <c r="B68" t="n">
         <v>67</v>
       </c>
       <c r="C68" t="n">
-        <v>1370.47</v>
+        <v>1371.11</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>Cabo Verde</t>
+          <t>United Arab Emirates</t>
         </is>
       </c>
       <c r="B69" t="n">
         <v>68</v>
       </c>
       <c r="C69" t="n">
-        <v>1369.29</v>
+        <v>1370.47</v>
       </c>
     </row>
     <row r="70">
@@ -2597,7 +2597,7 @@
         <v>70</v>
       </c>
       <c r="C71" t="n">
-        <v>1366.56</v>
+        <v>1365.3</v>
       </c>
     </row>
     <row r="72">
@@ -2649,7 +2649,7 @@
         <v>74</v>
       </c>
       <c r="C75" t="n">
-        <v>1343.92</v>
+        <v>1342.77</v>
       </c>
     </row>
     <row r="76">
@@ -2688,7 +2688,7 @@
         <v>77</v>
       </c>
       <c r="C78" t="n">
-        <v>1329.42</v>
+        <v>1326</v>
       </c>
     </row>
     <row r="79">
@@ -2701,7 +2701,7 @@
         <v>78</v>
       </c>
       <c r="C79" t="n">
-        <v>1317.17</v>
+        <v>1319.12</v>
       </c>
     </row>
     <row r="80">
@@ -2746,27 +2746,27 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>Haiti</t>
+          <t>Curaçao</t>
         </is>
       </c>
       <c r="B83" t="n">
         <v>82</v>
       </c>
       <c r="C83" t="n">
-        <v>1293.1</v>
+        <v>1294.77</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>Curaçao</t>
+          <t>Haiti</t>
         </is>
       </c>
       <c r="B84" t="n">
         <v>83</v>
       </c>
       <c r="C84" t="n">
-        <v>1293.08</v>
+        <v>1293.1</v>
       </c>
     </row>
     <row r="85">
@@ -2792,7 +2792,7 @@
         <v>85</v>
       </c>
       <c r="C86" t="n">
-        <v>1276.66</v>
+        <v>1275.58</v>
       </c>
     </row>
     <row r="87">
@@ -2824,79 +2824,79 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>Uganda</t>
+          <t>Angola</t>
         </is>
       </c>
       <c r="B89" t="n">
         <v>88</v>
       </c>
       <c r="C89" t="n">
-        <v>1264.09</v>
+        <v>1265.58</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>Angola</t>
+          <t>Uganda</t>
         </is>
       </c>
       <c r="B90" t="n">
         <v>89</v>
       </c>
       <c r="C90" t="n">
-        <v>1262.22</v>
+        <v>1264.09</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>Benin</t>
+          <t>Zambia</t>
         </is>
       </c>
       <c r="B91" t="n">
         <v>90</v>
       </c>
       <c r="C91" t="n">
-        <v>1258.22</v>
+        <v>1255.82</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>Zambia</t>
+          <t>China PR</t>
         </is>
       </c>
       <c r="B92" t="n">
         <v>91</v>
       </c>
       <c r="C92" t="n">
-        <v>1255.82</v>
+        <v>1254.81</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>China PR</t>
+          <t>Bahrain</t>
         </is>
       </c>
       <c r="B93" t="n">
         <v>92</v>
       </c>
       <c r="C93" t="n">
-        <v>1254.85</v>
+        <v>1254.41</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>Bahrain</t>
+          <t>Benin</t>
         </is>
       </c>
       <c r="B94" t="n">
         <v>93</v>
       </c>
       <c r="C94" t="n">
-        <v>1254.41</v>
+        <v>1252.17</v>
       </c>
     </row>
     <row r="95">
@@ -2909,7 +2909,7 @@
         <v>94</v>
       </c>
       <c r="C95" t="n">
-        <v>1250.76</v>
+        <v>1250.8</v>
       </c>
     </row>
     <row r="96">
@@ -2922,7 +2922,7 @@
         <v>95</v>
       </c>
       <c r="C96" t="n">
-        <v>1244.73</v>
+        <v>1243.71</v>
       </c>
     </row>
     <row r="97">
@@ -2935,7 +2935,7 @@
         <v>96</v>
       </c>
       <c r="C97" t="n">
-        <v>1241.32</v>
+        <v>1242.88</v>
       </c>
     </row>
     <row r="98">
@@ -2948,7 +2948,7 @@
         <v>97</v>
       </c>
       <c r="C98" t="n">
-        <v>1240.78</v>
+        <v>1238.74</v>
       </c>
     </row>
     <row r="99">
@@ -2961,7 +2961,7 @@
         <v>98</v>
       </c>
       <c r="C99" t="n">
-        <v>1226.36</v>
+        <v>1232.82</v>
       </c>
     </row>
     <row r="100">
@@ -2980,53 +2980,53 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>Tajikistan</t>
+          <t>El Salvador</t>
         </is>
       </c>
       <c r="B101" t="n">
         <v>100</v>
       </c>
       <c r="C101" t="n">
-        <v>1225.52</v>
+        <v>1225.34</v>
       </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>Mozambique</t>
+          <t>Tajikistan</t>
         </is>
       </c>
       <c r="B102" t="n">
         <v>101</v>
       </c>
       <c r="C102" t="n">
-        <v>1224.31</v>
+        <v>1224.19</v>
       </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>El Salvador</t>
+          <t>Trinidad and Tobago</t>
         </is>
       </c>
       <c r="B103" t="n">
         <v>102</v>
       </c>
       <c r="C103" t="n">
-        <v>1223.28</v>
+        <v>1219.59</v>
       </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>Trinidad and Tobago</t>
+          <t>Mozambique</t>
         </is>
       </c>
       <c r="B104" t="n">
         <v>103</v>
       </c>
       <c r="C104" t="n">
-        <v>1221.95</v>
+        <v>1218.62</v>
       </c>
     </row>
     <row r="105">
@@ -3058,27 +3058,27 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>Armenia</t>
+          <t>Kyrgyz Republic</t>
         </is>
       </c>
       <c r="B107" t="n">
         <v>106</v>
       </c>
       <c r="C107" t="n">
-        <v>1191.33</v>
+        <v>1192.16</v>
       </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>Kyrgyz Republic</t>
+          <t>Armenia</t>
         </is>
       </c>
       <c r="B108" t="n">
         <v>107</v>
       </c>
       <c r="C108" t="n">
-        <v>1191.14</v>
+        <v>1189.63</v>
       </c>
     </row>
     <row r="109">
@@ -3097,14 +3097,14 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>Kazakhstan</t>
+          <t>Kenya</t>
         </is>
       </c>
       <c r="B110" t="n">
         <v>109</v>
       </c>
       <c r="C110" t="n">
-        <v>1183.04</v>
+        <v>1185.08</v>
       </c>
     </row>
     <row r="111">
@@ -3123,66 +3123,66 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>Kenya</t>
+          <t>Kazakhstan</t>
         </is>
       </c>
       <c r="B112" t="n">
         <v>111</v>
       </c>
       <c r="C112" t="n">
-        <v>1181.14</v>
+        <v>1180.78</v>
       </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>Niger</t>
+          <t>Tanzania</t>
         </is>
       </c>
       <c r="B113" t="n">
         <v>112</v>
       </c>
       <c r="C113" t="n">
-        <v>1180.42</v>
+        <v>1180.27</v>
       </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>Tanzania</t>
+          <t>Mauritania</t>
         </is>
       </c>
       <c r="B114" t="n">
         <v>113</v>
       </c>
       <c r="C114" t="n">
-        <v>1180.27</v>
+        <v>1176.68</v>
       </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>Lebanon</t>
+          <t>Niger</t>
         </is>
       </c>
       <c r="B115" t="n">
         <v>114</v>
       </c>
       <c r="C115" t="n">
-        <v>1172.22</v>
+        <v>1175.33</v>
       </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>Mauritania</t>
+          <t>Lebanon</t>
         </is>
       </c>
       <c r="B116" t="n">
         <v>115</v>
       </c>
       <c r="C116" t="n">
-        <v>1171.6</v>
+        <v>1172.22</v>
       </c>
     </row>
     <row r="117">
@@ -3221,33 +3221,33 @@
         <v>118</v>
       </c>
       <c r="C119" t="n">
-        <v>1151.45</v>
+        <v>1157.14</v>
       </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>Korea DPR</t>
+          <t>Togo</t>
         </is>
       </c>
       <c r="B120" t="n">
         <v>119</v>
       </c>
       <c r="C120" t="n">
-        <v>1151.05</v>
+        <v>1152.76</v>
       </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>Sierra Leone</t>
+          <t>Korea DPR</t>
         </is>
       </c>
       <c r="B121" t="n">
         <v>120</v>
       </c>
       <c r="C121" t="n">
-        <v>1148.98</v>
+        <v>1151.05</v>
       </c>
     </row>
     <row r="122">
@@ -3266,14 +3266,14 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>Togo</t>
+          <t>Sierra Leone</t>
         </is>
       </c>
       <c r="B123" t="n">
         <v>122</v>
       </c>
       <c r="C123" t="n">
-        <v>1146.7</v>
+        <v>1147.56</v>
       </c>
     </row>
     <row r="124">
@@ -3286,33 +3286,33 @@
         <v>123</v>
       </c>
       <c r="C124" t="n">
-        <v>1137.14</v>
+        <v>1136.59</v>
       </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>Suriname</t>
+          <t>Cyprus</t>
         </is>
       </c>
       <c r="B125" t="n">
         <v>124</v>
       </c>
       <c r="C125" t="n">
-        <v>1132.43</v>
+        <v>1133.25</v>
       </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>Cyprus</t>
+          <t>Suriname</t>
         </is>
       </c>
       <c r="B126" t="n">
         <v>125</v>
       </c>
       <c r="C126" t="n">
-        <v>1131.06</v>
+        <v>1132.43</v>
       </c>
     </row>
     <row r="127">
@@ -3325,20 +3325,20 @@
         <v>126</v>
       </c>
       <c r="C127" t="n">
-        <v>1130.26</v>
+        <v>1132</v>
       </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>Malawi</t>
+          <t>Estonia</t>
         </is>
       </c>
       <c r="B128" t="n">
         <v>127</v>
       </c>
       <c r="C128" t="n">
-        <v>1128.03</v>
+        <v>1130.64</v>
       </c>
     </row>
     <row r="129">
@@ -3357,14 +3357,14 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>Estonia</t>
+          <t>Malawi</t>
         </is>
       </c>
       <c r="B130" t="n">
         <v>129</v>
       </c>
       <c r="C130" t="n">
-        <v>1121.1</v>
+        <v>1122.05</v>
       </c>
     </row>
     <row r="131">
@@ -3442,59 +3442,59 @@
         <v>135</v>
       </c>
       <c r="C136" t="n">
-        <v>1096.73</v>
+        <v>1100.95</v>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>Latvia</t>
+          <t>Malaysia</t>
         </is>
       </c>
       <c r="B137" t="n">
         <v>136</v>
       </c>
       <c r="C137" t="n">
-        <v>1090.57</v>
+        <v>1086.22</v>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>Malaysia</t>
+          <t>Latvia</t>
         </is>
       </c>
       <c r="B138" t="n">
         <v>137</v>
       </c>
       <c r="C138" t="n">
-        <v>1086.22</v>
+        <v>1085.66</v>
       </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>Central African Republic</t>
+          <t>India</t>
         </is>
       </c>
       <c r="B139" t="n">
         <v>138</v>
       </c>
       <c r="C139" t="n">
-        <v>1084.18</v>
+        <v>1084.93</v>
       </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>India</t>
+          <t>Central African Republic</t>
         </is>
       </c>
       <c r="B140" t="n">
         <v>139</v>
       </c>
       <c r="C140" t="n">
-        <v>1083.6</v>
+        <v>1080.82</v>
       </c>
     </row>
     <row r="141">
@@ -3507,7 +3507,7 @@
         <v>140</v>
       </c>
       <c r="C141" t="n">
-        <v>1079.02</v>
+        <v>1080.44</v>
       </c>
     </row>
     <row r="142">
@@ -3539,53 +3539,53 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>Dominican Republic</t>
+          <t>Ethiopia</t>
         </is>
       </c>
       <c r="B144" t="n">
         <v>143</v>
       </c>
       <c r="C144" t="n">
-        <v>1076.5</v>
+        <v>1077.52</v>
       </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>Ethiopia</t>
+          <t>Dominican Republic</t>
         </is>
       </c>
       <c r="B145" t="n">
         <v>144</v>
       </c>
       <c r="C145" t="n">
-        <v>1071.55</v>
+        <v>1076.5</v>
       </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>Lesotho</t>
+          <t>Yemen</t>
         </is>
       </c>
       <c r="B146" t="n">
         <v>145</v>
       </c>
       <c r="C146" t="n">
-        <v>1068.22</v>
+        <v>1065.24</v>
       </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>Yemen</t>
+          <t>Lesotho</t>
         </is>
       </c>
       <c r="B147" t="n">
         <v>146</v>
       </c>
       <c r="C147" t="n">
-        <v>1065.24</v>
+        <v>1064.29</v>
       </c>
     </row>
     <row r="148">
@@ -3604,27 +3604,27 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>Lithuania</t>
+          <t>Singapore</t>
         </is>
       </c>
       <c r="B149" t="n">
         <v>148</v>
       </c>
       <c r="C149" t="n">
-        <v>1058.42</v>
+        <v>1057.95</v>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>Singapore</t>
+          <t>Lithuania</t>
         </is>
       </c>
       <c r="B150" t="n">
         <v>149</v>
       </c>
       <c r="C150" t="n">
-        <v>1057.95</v>
+        <v>1056.85</v>
       </c>
     </row>
     <row r="151">
@@ -3682,14 +3682,14 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>Hong Kong, China</t>
+          <t>Puerto Rico</t>
         </is>
       </c>
       <c r="B155" t="n">
         <v>154</v>
       </c>
       <c r="C155" t="n">
-        <v>1030.24</v>
+        <v>1024.3</v>
       </c>
     </row>
     <row r="156">
@@ -3702,20 +3702,20 @@
         <v>155</v>
       </c>
       <c r="C156" t="n">
-        <v>1024.38</v>
+        <v>1024.17</v>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>Puerto Rico</t>
+          <t>Hong Kong, China</t>
         </is>
       </c>
       <c r="B157" t="n">
         <v>156</v>
       </c>
       <c r="C157" t="n">
-        <v>1024.3</v>
+        <v>1024.16</v>
       </c>
     </row>
     <row r="158">
@@ -3741,7 +3741,7 @@
         <v>158</v>
       </c>
       <c r="C159" t="n">
-        <v>1011.88</v>
+        <v>1010.91</v>
       </c>
     </row>
     <row r="160">
@@ -3754,7 +3754,7 @@
         <v>159</v>
       </c>
       <c r="C160" t="n">
-        <v>1006.54</v>
+        <v>1008.24</v>
       </c>
     </row>
     <row r="161">
@@ -3767,7 +3767,7 @@
         <v>160</v>
       </c>
       <c r="C161" t="n">
-        <v>1002.32</v>
+        <v>1002.53</v>
       </c>
     </row>
     <row r="162">
@@ -3838,14 +3838,14 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>Afghanistan</t>
+          <t>St Lucia</t>
         </is>
       </c>
       <c r="B167" t="n">
         <v>166</v>
       </c>
       <c r="C167" t="n">
-        <v>977.5700000000001</v>
+        <v>976.71</v>
       </c>
     </row>
     <row r="168">
@@ -3858,59 +3858,59 @@
         <v>167</v>
       </c>
       <c r="C168" t="n">
-        <v>976.87</v>
+        <v>975.05</v>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>St Lucia</t>
+          <t>Papua New Guinea</t>
         </is>
       </c>
       <c r="B169" t="n">
         <v>168</v>
       </c>
       <c r="C169" t="n">
-        <v>976.71</v>
+        <v>974.9</v>
       </c>
     </row>
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>Papua New Guinea</t>
+          <t>South Sudan</t>
         </is>
       </c>
       <c r="B170" t="n">
         <v>169</v>
       </c>
       <c r="C170" t="n">
-        <v>974.9</v>
+        <v>970.9400000000001</v>
       </c>
     </row>
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>South Sudan</t>
+          <t>St Vincent and the Grenadines</t>
         </is>
       </c>
       <c r="B171" t="n">
         <v>170</v>
       </c>
       <c r="C171" t="n">
-        <v>970.9400000000001</v>
+        <v>968.27</v>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>St Vincent and the Grenadines</t>
+          <t>Afghanistan</t>
         </is>
       </c>
       <c r="B172" t="n">
         <v>171</v>
       </c>
       <c r="C172" t="n">
-        <v>968.27</v>
+        <v>968.0700000000001</v>
       </c>
     </row>
     <row r="173">
@@ -3923,7 +3923,7 @@
         <v>172</v>
       </c>
       <c r="C173" t="n">
-        <v>948.38</v>
+        <v>946.4299999999999</v>
       </c>
     </row>
     <row r="174">
@@ -3955,27 +3955,27 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>Montserrat</t>
+          <t>Cambodia</t>
         </is>
       </c>
       <c r="B176" t="n">
         <v>175</v>
       </c>
       <c r="C176" t="n">
-        <v>916.75</v>
+        <v>922.3200000000001</v>
       </c>
     </row>
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>Cambodia</t>
+          <t>Montserrat</t>
         </is>
       </c>
       <c r="B177" t="n">
         <v>176</v>
       </c>
       <c r="C177" t="n">
-        <v>916.24</v>
+        <v>916.75</v>
       </c>
     </row>
     <row r="178">
@@ -4111,14 +4111,14 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>Aruba</t>
+          <t>Sri Lanka</t>
         </is>
       </c>
       <c r="B188" t="n">
         <v>187</v>
       </c>
       <c r="C188" t="n">
-        <v>877.3</v>
+        <v>876.86</v>
       </c>
     </row>
     <row r="189">
@@ -4137,14 +4137,14 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>Bhutan</t>
+          <t>Aruba</t>
         </is>
       </c>
       <c r="B190" t="n">
         <v>189</v>
       </c>
       <c r="C190" t="n">
-        <v>875.85</v>
+        <v>875.61</v>
       </c>
     </row>
     <row r="191">
@@ -4163,131 +4163,131 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>Sri Lanka</t>
+          <t>American Samoa</t>
         </is>
       </c>
       <c r="B192" t="n">
         <v>191</v>
       </c>
       <c r="C192" t="n">
-        <v>871.8200000000001</v>
+        <v>871.61</v>
       </c>
     </row>
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>American Samoa</t>
+          <t>Bhutan</t>
         </is>
       </c>
       <c r="B193" t="n">
         <v>192</v>
       </c>
       <c r="C193" t="n">
-        <v>871.61</v>
+        <v>870.8099999999999</v>
       </c>
     </row>
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>Brunei Darussalam</t>
+          <t>Macau</t>
         </is>
       </c>
       <c r="B194" t="n">
         <v>193</v>
       </c>
       <c r="C194" t="n">
-        <v>863.09</v>
+        <v>858.03</v>
       </c>
     </row>
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>Macau</t>
+          <t>Brunei Darussalam</t>
         </is>
       </c>
       <c r="B195" t="n">
         <v>194</v>
       </c>
       <c r="C195" t="n">
-        <v>858.03</v>
+        <v>857.73</v>
       </c>
     </row>
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>Cayman Islands</t>
+          <t>São Tomé and Príncipe</t>
         </is>
       </c>
       <c r="B196" t="n">
         <v>195</v>
       </c>
       <c r="C196" t="n">
-        <v>855.45</v>
+        <v>855.4400000000001</v>
       </c>
     </row>
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>São Tomé and Príncipe</t>
+          <t>Djibouti</t>
         </is>
       </c>
       <c r="B197" t="n">
         <v>196</v>
       </c>
       <c r="C197" t="n">
-        <v>855.4400000000001</v>
+        <v>853.58</v>
       </c>
     </row>
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>Djibouti</t>
+          <t>Cayman Islands</t>
         </is>
       </c>
       <c r="B198" t="n">
         <v>197</v>
       </c>
       <c r="C198" t="n">
-        <v>853.58</v>
+        <v>850.0599999999999</v>
       </c>
     </row>
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
-          <t>Somalia</t>
+          <t>Pakistan</t>
         </is>
       </c>
       <c r="B199" t="n">
         <v>198</v>
       </c>
       <c r="C199" t="n">
-        <v>839.17</v>
+        <v>840.28</v>
       </c>
     </row>
     <row r="200">
       <c r="A200" t="inlineStr">
         <is>
-          <t>Tonga</t>
+          <t>Somalia</t>
         </is>
       </c>
       <c r="B200" t="n">
         <v>199</v>
       </c>
       <c r="C200" t="n">
-        <v>835.64</v>
+        <v>839.17</v>
       </c>
     </row>
     <row r="201">
       <c r="A201" t="inlineStr">
         <is>
-          <t>Pakistan</t>
+          <t>Tonga</t>
         </is>
       </c>
       <c r="B201" t="n">
         <v>200</v>
       </c>
       <c r="C201" t="n">
-        <v>830.78</v>
+        <v>835.64</v>
       </c>
     </row>
     <row r="202">
@@ -4300,33 +4300,33 @@
         <v>201</v>
       </c>
       <c r="C202" t="n">
-        <v>825.64</v>
+        <v>831</v>
       </c>
     </row>
     <row r="203">
       <c r="A203" t="inlineStr">
         <is>
-          <t>Guam</t>
+          <t>Gibraltar</t>
         </is>
       </c>
       <c r="B203" t="n">
         <v>202</v>
       </c>
       <c r="C203" t="n">
-        <v>822.8</v>
+        <v>820.26</v>
       </c>
     </row>
     <row r="204">
       <c r="A204" t="inlineStr">
         <is>
-          <t>Gibraltar</t>
+          <t>Guam</t>
         </is>
       </c>
       <c r="B204" t="n">
         <v>203</v>
       </c>
       <c r="C204" t="n">
-        <v>814.87</v>
+        <v>819.54</v>
       </c>
     </row>
     <row r="205">
@@ -4365,7 +4365,7 @@
         <v>206</v>
       </c>
       <c r="C207" t="n">
-        <v>799.89</v>
+        <v>797.7</v>
       </c>
     </row>
     <row r="208">
@@ -4430,7 +4430,7 @@
         <v>211</v>
       </c>
       <c r="C212" t="n">
-        <v>722.9299999999999</v>
+        <v>721.2</v>
       </c>
     </row>
   </sheetData>

</xml_diff>